<commit_message>
Use «شاشة ١ / شاشة ٢» labels (statics, Kafu ep3, content plan)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012aeGc1ksmT1Mdqdqyz4pXR
</commit_message>
<xml_diff>
--- a/content-plan/PopupPush_جدول_المحتوى_العضوي.xlsx
+++ b/content-plan/PopupPush_جدول_المحتوى_العضوي.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="H3" s="27" t="inlineStr">
         <is>
-          <t>قناة ١ على شاشة، قناة ٢ على ثانية، والعرض على الكل… وكل هذا من جوالك 📲
+          <t>شاشة ١ على شاشة، شاشة ٢ على ثانية، والعرض على الكل… وكل هذا من جوالك 📲
 PopupPush يتحكم بماتريكس المحل، يبدّل القنوات، وينزّل العروض — بدون ريموت ولا لف بين الشاشات.
 مقهى أو لاونج؟ راسلنا واتساب — الرابط بالبايو.</t>
         </is>
@@ -918,13 +918,13 @@
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>قناة ١ هنا… وقناة ٢ هناك | أبشر، خلّها على كفو!</t>
+          <t>شاشة ١ هنا… وشاشة ٢ هناك | أبشر، خلّها على كفو!</t>
         </is>
       </c>
       <c r="H7" s="27" t="inlineStr">
         <is>
           <t>ماتشين بنفس الوقت؟ ولا يهمك 😎
-كفو يوزّع القنوات على الشاشات من الجوال: هذي قناة ١، وهذي قناة ٢ — بدون ما تدوّر على ريموت.
+كفو يوزّع القنوات على الشاشات من الجوال: هذي شاشة ١، وهذي شاشة ٢ — بدون ما تدوّر على ريموت.
 #يوميات_كفو — الحلقة ٣ 🎬</t>
         </is>
       </c>

</xml_diff>